<commit_message>
Added drag times column
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/Research/variables/Variable Definitions RQ8_PH2_APR26.xlsx
+++ b/dashboard-ui/src/components/Research/variables/Variable Definitions RQ8_PH2_APR26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gary.cheng_cn\Projects\itm-evaluation-dashboard\dashboard-ui\src\components\Research\variables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF289364-23E6-4F45-8B29-D0BBEC1FAD13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B1289F-9DE2-44CC-BFD3-87B09A2BECE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="235">
   <si>
     <t>Variables</t>
   </si>
@@ -755,6 +755,18 @@
   </si>
   <si>
     <t>Urban Probe_SS1</t>
+  </si>
+  <si>
+    <t>Desert Patient{N}_drag_times</t>
+  </si>
+  <si>
+    <t>Comma-separated list of drag start timestamps</t>
+  </si>
+  <si>
+    <t>time(s)</t>
+  </si>
+  <si>
+    <t>Urban Patient{N}_drag_times</t>
   </si>
 </sst>
 </file>
@@ -1195,7 +1207,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:DX6"/>
+  <dimension ref="A1:DZ6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="16.7265625" style="2" bestFit="1" customWidth="1"/>
@@ -1219,32 +1231,32 @@
     <col min="58" max="65" width="16.7265625" style="10" customWidth="1"/>
     <col min="66" max="70" width="13" style="10" bestFit="1" customWidth="1"/>
     <col min="71" max="76" width="13" style="12" bestFit="1" customWidth="1"/>
-    <col min="77" max="85" width="13" style="12" customWidth="1"/>
-    <col min="86" max="91" width="13" style="10" bestFit="1" customWidth="1"/>
-    <col min="92" max="100" width="13" style="10" customWidth="1"/>
-    <col min="101" max="101" width="87.7265625" style="8" customWidth="1"/>
-    <col min="102" max="103" width="73" style="8" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="38.54296875" style="6" customWidth="1"/>
-    <col min="105" max="105" width="34.7265625" style="6" customWidth="1"/>
-    <col min="106" max="106" width="73" style="8" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="32.54296875" style="6" customWidth="1"/>
-    <col min="108" max="112" width="32.26953125" style="6" customWidth="1"/>
-    <col min="113" max="113" width="87.7265625" style="17" customWidth="1"/>
-    <col min="114" max="115" width="73" style="17" bestFit="1" customWidth="1"/>
-    <col min="116" max="116" width="38.54296875" style="15" customWidth="1"/>
-    <col min="117" max="117" width="34.7265625" style="15" customWidth="1"/>
-    <col min="118" max="118" width="73" style="17" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="87.7265625" style="17" customWidth="1"/>
-    <col min="120" max="121" width="73" style="17" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="38.54296875" style="15" customWidth="1"/>
-    <col min="123" max="123" width="34.7265625" style="15" customWidth="1"/>
-    <col min="124" max="124" width="73" style="17" bestFit="1" customWidth="1"/>
-    <col min="125" max="125" width="14.7265625" style="5" customWidth="1"/>
-    <col min="126" max="126" width="15.26953125" style="5" customWidth="1"/>
-    <col min="127" max="128" width="9.1796875" style="5"/>
+    <col min="77" max="86" width="13" style="12" customWidth="1"/>
+    <col min="87" max="92" width="13" style="10" bestFit="1" customWidth="1"/>
+    <col min="93" max="102" width="13" style="10" customWidth="1"/>
+    <col min="103" max="103" width="87.7265625" style="8" customWidth="1"/>
+    <col min="104" max="105" width="73" style="8" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="38.54296875" style="6" customWidth="1"/>
+    <col min="107" max="107" width="34.7265625" style="6" customWidth="1"/>
+    <col min="108" max="108" width="73" style="8" bestFit="1" customWidth="1"/>
+    <col min="109" max="109" width="32.54296875" style="6" customWidth="1"/>
+    <col min="110" max="114" width="32.26953125" style="6" customWidth="1"/>
+    <col min="115" max="115" width="87.7265625" style="17" customWidth="1"/>
+    <col min="116" max="117" width="73" style="17" bestFit="1" customWidth="1"/>
+    <col min="118" max="118" width="38.54296875" style="15" customWidth="1"/>
+    <col min="119" max="119" width="34.7265625" style="15" customWidth="1"/>
+    <col min="120" max="120" width="73" style="17" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="87.7265625" style="17" customWidth="1"/>
+    <col min="122" max="123" width="73" style="17" bestFit="1" customWidth="1"/>
+    <col min="124" max="124" width="38.54296875" style="15" customWidth="1"/>
+    <col min="125" max="125" width="34.7265625" style="15" customWidth="1"/>
+    <col min="126" max="126" width="73" style="17" bestFit="1" customWidth="1"/>
+    <col min="127" max="127" width="14.7265625" style="5" customWidth="1"/>
+    <col min="128" max="128" width="15.26953125" style="5" customWidth="1"/>
+    <col min="129" max="130" width="9.1796875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:128" s="3" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:130" s="3" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1477,160 +1489,166 @@
         <v>220</v>
       </c>
       <c r="BZ1" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="CA1" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="CA1" s="11" t="s">
+      <c r="CB1" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="CB1" s="11" t="s">
+      <c r="CC1" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="CC1" s="11" t="s">
+      <c r="CD1" s="11" t="s">
         <v>184</v>
       </c>
-      <c r="CD1" s="11" t="s">
+      <c r="CE1" s="11" t="s">
         <v>185</v>
       </c>
-      <c r="CE1" s="11" t="s">
+      <c r="CF1" s="11" t="s">
         <v>186</v>
       </c>
-      <c r="CF1" s="11" t="s">
+      <c r="CG1" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="CG1" s="11" t="s">
+      <c r="CH1" s="11" t="s">
         <v>188</v>
       </c>
-      <c r="CH1" s="9" t="s">
+      <c r="CI1" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="CI1" s="9" t="s">
+      <c r="CJ1" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="CJ1" s="9" t="s">
+      <c r="CK1" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="CK1" s="9" t="s">
+      <c r="CL1" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="CL1" s="9" t="s">
+      <c r="CM1" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="CM1" s="9" t="s">
+      <c r="CN1" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="CN1" s="9" t="s">
+      <c r="CO1" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="CO1" s="9" t="s">
+      <c r="CP1" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="CQ1" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="CP1" s="9" t="s">
+      <c r="CR1" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="CQ1" s="9" t="s">
+      <c r="CS1" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="CR1" s="9" t="s">
+      <c r="CT1" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="CS1" s="9" t="s">
+      <c r="CU1" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="CT1" s="9" t="s">
+      <c r="CV1" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="CU1" s="9" t="s">
+      <c r="CW1" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="CV1" s="9" t="s">
+      <c r="CX1" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="CW1" s="6" t="s">
+      <c r="CY1" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="CX1" s="6" t="s">
+      <c r="CZ1" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="CY1" s="6" t="s">
+      <c r="DA1" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="CZ1" s="6" t="s">
+      <c r="DB1" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="DA1" s="6" t="s">
+      <c r="DC1" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="DB1" s="6" t="s">
+      <c r="DD1" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="DC1" s="6" t="s">
+      <c r="DE1" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="DD1" s="6" t="s">
+      <c r="DF1" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="DE1" s="6" t="s">
+      <c r="DG1" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="DF1" s="6" t="s">
+      <c r="DH1" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="DG1" s="6" t="s">
+      <c r="DI1" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="DH1" s="6" t="s">
+      <c r="DJ1" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="DI1" s="15" t="s">
+      <c r="DK1" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="DJ1" s="15" t="s">
+      <c r="DL1" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="DK1" s="15" t="s">
+      <c r="DM1" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="DL1" s="15" t="s">
+      <c r="DN1" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="DM1" s="15" t="s">
+      <c r="DO1" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="DN1" s="15" t="s">
+      <c r="DP1" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="DO1" s="15" t="s">
+      <c r="DQ1" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="DP1" s="15" t="s">
+      <c r="DR1" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="DQ1" s="15" t="s">
+      <c r="DS1" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="DR1" s="15" t="s">
+      <c r="DT1" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="DS1" s="15" t="s">
+      <c r="DU1" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="DT1" s="15" t="s">
+      <c r="DV1" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="DU1" s="4" t="s">
+      <c r="DW1" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="DV1" s="4" t="s">
+      <c r="DX1" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="DW1" s="4" t="s">
+      <c r="DY1" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="DX1" s="4" t="s">
+      <c r="DZ1" s="4" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="2" spans="1:128" s="3" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:130" s="3" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>82</v>
       </c>
@@ -1886,7 +1904,7 @@
       <c r="CG2" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="CH2" s="9" t="s">
+      <c r="CH2" s="11" t="s">
         <v>85</v>
       </c>
       <c r="CI2" s="9" t="s">
@@ -1931,11 +1949,11 @@
       <c r="CV2" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="CW2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="CX2" s="7" t="s">
-        <v>86</v>
+      <c r="CW2" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="CX2" s="9" t="s">
+        <v>85</v>
       </c>
       <c r="CY2" s="7" t="s">
         <v>86</v>
@@ -1967,11 +1985,11 @@
       <c r="DH2" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="DI2" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="DJ2" s="16" t="s">
-        <v>87</v>
+      <c r="DI2" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="DJ2" s="7" t="s">
+        <v>86</v>
       </c>
       <c r="DK2" s="16" t="s">
         <v>87</v>
@@ -2003,11 +2021,11 @@
       <c r="DT2" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="DU2" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="DV2" s="4" t="s">
-        <v>149</v>
+      <c r="DU2" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="DV2" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="DW2" s="4" t="s">
         <v>149</v>
@@ -2015,8 +2033,14 @@
       <c r="DX2" s="4" t="s">
         <v>149</v>
       </c>
+      <c r="DY2" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="DZ2" s="4" t="s">
+        <v>149</v>
+      </c>
     </row>
-    <row r="3" spans="1:128" s="3" customFormat="1" ht="299" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:130" s="3" customFormat="1" ht="299" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>88</v>
       </c>
@@ -2249,160 +2273,166 @@
         <v>216</v>
       </c>
       <c r="BZ3" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="CA3" s="11" t="s">
         <v>206</v>
       </c>
-      <c r="CA3" s="11" t="s">
+      <c r="CB3" s="11" t="s">
         <v>207</v>
       </c>
-      <c r="CB3" s="11" t="s">
+      <c r="CC3" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="CC3" s="11" t="s">
+      <c r="CD3" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="CD3" s="11" t="s">
+      <c r="CE3" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="CE3" s="11" t="s">
+      <c r="CF3" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="CF3" s="11" t="s">
+      <c r="CG3" s="11" t="s">
         <v>212</v>
       </c>
-      <c r="CG3" s="11" t="s">
+      <c r="CH3" s="11" t="s">
         <v>213</v>
       </c>
-      <c r="CH3" s="9" t="s">
+      <c r="CI3" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="CI3" s="9" t="s">
+      <c r="CJ3" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="CJ3" s="9" t="s">
+      <c r="CK3" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="CK3" s="9" t="s">
+      <c r="CL3" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="CL3" s="9" t="s">
+      <c r="CM3" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="CM3" s="9" t="s">
+      <c r="CN3" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="CN3" s="9" t="s">
+      <c r="CO3" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="CO3" s="9" t="s">
+      <c r="CP3" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="CQ3" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="CP3" s="9" t="s">
+      <c r="CR3" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="CQ3" s="9" t="s">
+      <c r="CS3" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="CR3" s="9" t="s">
+      <c r="CT3" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="CS3" s="9" t="s">
+      <c r="CU3" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="CT3" s="9" t="s">
+      <c r="CV3" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="CU3" s="9" t="s">
+      <c r="CW3" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="CV3" s="9" t="s">
+      <c r="CX3" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="CW3" s="7" t="s">
+      <c r="CY3" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="CX3" s="7" t="s">
+      <c r="CZ3" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="CY3" s="7" t="s">
+      <c r="DA3" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="CZ3" s="7" t="s">
+      <c r="DB3" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="DA3" s="7" t="s">
+      <c r="DC3" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="DB3" s="7" t="s">
+      <c r="DD3" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="DC3" s="7" t="s">
+      <c r="DE3" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="DD3" s="7" t="s">
+      <c r="DF3" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="DE3" s="7" t="s">
+      <c r="DG3" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="DF3" s="7" t="s">
+      <c r="DH3" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="DG3" s="7" t="s">
+      <c r="DI3" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="DH3" s="7" t="s">
+      <c r="DJ3" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="DI3" s="16" t="s">
+      <c r="DK3" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="DJ3" s="16" t="s">
+      <c r="DL3" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="DK3" s="16" t="s">
+      <c r="DM3" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="DL3" s="16" t="s">
+      <c r="DN3" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="DM3" s="16" t="s">
+      <c r="DO3" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="DN3" s="16" t="s">
+      <c r="DP3" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="DO3" s="16" t="s">
+      <c r="DQ3" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="DP3" s="16" t="s">
+      <c r="DR3" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="DQ3" s="16" t="s">
+      <c r="DS3" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="DR3" s="16" t="s">
+      <c r="DT3" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="DS3" s="16" t="s">
+      <c r="DU3" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="DT3" s="16" t="s">
+      <c r="DV3" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="DU3" s="4" t="s">
+      <c r="DW3" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="DV3" s="4" t="s">
+      <c r="DX3" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="DW3" s="4" t="s">
+      <c r="DY3" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="DX3" s="4" t="s">
+      <c r="DZ3" s="4" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="4" spans="1:128" s="3" customFormat="1" ht="100.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:130" s="3" customFormat="1" ht="100.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>125</v>
       </c>
@@ -2633,7 +2663,7 @@
         <v>217</v>
       </c>
       <c r="BZ4" s="11" t="s">
-        <v>131</v>
+        <v>233</v>
       </c>
       <c r="CA4" s="11" t="s">
         <v>131</v>
@@ -2656,32 +2686,32 @@
       <c r="CG4" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="CH4" s="9" t="s">
+      <c r="CH4" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="CI4" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="CI4" s="9" t="s">
-        <v>131</v>
-      </c>
       <c r="CJ4" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="CK4" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="CK4" s="9" t="s">
-        <v>131</v>
-      </c>
       <c r="CL4" s="9" t="s">
         <v>131</v>
       </c>
       <c r="CM4" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="CN4" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="CN4" s="9" t="s">
+      <c r="CO4" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="CO4" s="9" t="s">
-        <v>131</v>
-      </c>
       <c r="CP4" s="9" t="s">
-        <v>131</v>
+        <v>233</v>
       </c>
       <c r="CQ4" s="9" t="s">
         <v>131</v>
@@ -2701,8 +2731,12 @@
       <c r="CV4" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="CW4" s="7"/>
-      <c r="CX4" s="7"/>
+      <c r="CW4" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="CX4" s="9" t="s">
+        <v>131</v>
+      </c>
       <c r="CY4" s="7"/>
       <c r="CZ4" s="7"/>
       <c r="DA4" s="7"/>
@@ -2713,8 +2747,8 @@
       <c r="DF4" s="7"/>
       <c r="DG4" s="7"/>
       <c r="DH4" s="7"/>
-      <c r="DI4" s="16"/>
-      <c r="DJ4" s="16"/>
+      <c r="DI4" s="7"/>
+      <c r="DJ4" s="7"/>
       <c r="DK4" s="16"/>
       <c r="DL4" s="16"/>
       <c r="DM4" s="16"/>
@@ -2725,14 +2759,14 @@
       <c r="DR4" s="16"/>
       <c r="DS4" s="16"/>
       <c r="DT4" s="16"/>
-      <c r="DU4" s="4"/>
-      <c r="DV4" s="4"/>
+      <c r="DU4" s="16"/>
+      <c r="DV4" s="16"/>
       <c r="DW4" s="4"/>
       <c r="DX4" s="4"/>
+      <c r="DY4" s="4"/>
+      <c r="DZ4" s="4"/>
     </row>
-    <row r="5" spans="1:128" x14ac:dyDescent="0.35">
-      <c r="CW5" s="7"/>
-      <c r="CX5" s="7"/>
+    <row r="5" spans="1:130" x14ac:dyDescent="0.35">
       <c r="CY5" s="7"/>
       <c r="CZ5" s="7"/>
       <c r="DA5" s="7"/>
@@ -2743,8 +2777,8 @@
       <c r="DF5" s="7"/>
       <c r="DG5" s="7"/>
       <c r="DH5" s="7"/>
-      <c r="DI5" s="16"/>
-      <c r="DJ5" s="16"/>
+      <c r="DI5" s="7"/>
+      <c r="DJ5" s="7"/>
       <c r="DK5" s="16"/>
       <c r="DL5" s="16"/>
       <c r="DM5" s="16"/>
@@ -2755,10 +2789,10 @@
       <c r="DR5" s="16"/>
       <c r="DS5" s="16"/>
       <c r="DT5" s="16"/>
+      <c r="DU5" s="16"/>
+      <c r="DV5" s="16"/>
     </row>
-    <row r="6" spans="1:128" x14ac:dyDescent="0.35">
-      <c r="CW6" s="7"/>
-      <c r="CX6" s="7"/>
+    <row r="6" spans="1:130" x14ac:dyDescent="0.35">
       <c r="CY6" s="7"/>
       <c r="CZ6" s="7"/>
       <c r="DA6" s="7"/>
@@ -2769,8 +2803,8 @@
       <c r="DF6" s="7"/>
       <c r="DG6" s="7"/>
       <c r="DH6" s="7"/>
-      <c r="DI6" s="16"/>
-      <c r="DJ6" s="16"/>
+      <c r="DI6" s="7"/>
+      <c r="DJ6" s="7"/>
       <c r="DK6" s="16"/>
       <c r="DL6" s="16"/>
       <c r="DM6" s="16"/>
@@ -2781,6 +2815,8 @@
       <c r="DR6" s="16"/>
       <c r="DS6" s="16"/>
       <c r="DT6" s="16"/>
+      <c r="DU6" s="16"/>
+      <c r="DV6" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add missing kdmas and alignment scores
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/Research/variables/Variable Definitions RQ8_PH2_APR26.xlsx
+++ b/dashboard-ui/src/components/Research/variables/Variable Definitions RQ8_PH2_APR26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gary.cheng_cn\Projects\itm-evaluation-dashboard\dashboard-ui\src\components\Research\variables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B1289F-9DE2-44CC-BFD3-87B09A2BECE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C120C1-3157-4CC0-8B81-B1DDAF42F4E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RQ8" sheetId="1" r:id="rId1"/>
@@ -212,9 +212,6 @@
     <t>Urban Patient{N}_tag</t>
   </si>
   <si>
-    <t>AF_Intercept_Text</t>
-  </si>
-  <si>
     <t>AF_medical_Text</t>
   </si>
   <si>
@@ -248,9 +245,6 @@
     <t>SS_attribute_Text</t>
   </si>
   <si>
-    <t>AF_Intercept_Desert</t>
-  </si>
-  <si>
     <t>AF_medical_Desert</t>
   </si>
   <si>
@@ -264,9 +258,6 @@
   </si>
   <si>
     <t>MF_attribute_Desert</t>
-  </si>
-  <si>
-    <t>AF_Intercept_Urban</t>
   </si>
   <si>
     <t>AF_medical_Urban</t>
@@ -767,6 +758,15 @@
   </si>
   <si>
     <t>Urban Patient{N}_drag_times</t>
+  </si>
+  <si>
+    <t>AF_intercept_Text</t>
+  </si>
+  <si>
+    <t>AF_intercept_Desert</t>
+  </si>
+  <si>
+    <t>AF_intercept_Urban</t>
   </si>
 </sst>
 </file>
@@ -1267,10 +1267,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="F1" s="11" t="s">
         <v>3</v>
@@ -1303,16 +1303,16 @@
         <v>12</v>
       </c>
       <c r="P1" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="Q1" s="11" t="s">
         <v>221</v>
       </c>
-      <c r="Q1" s="11" t="s">
-        <v>224</v>
-      </c>
       <c r="R1" s="11" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="S1" s="11" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="T1" s="9" t="s">
         <v>13</v>
@@ -1342,10 +1342,10 @@
         <v>21</v>
       </c>
       <c r="AC1" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="AD1" s="9" t="s">
         <v>227</v>
-      </c>
-      <c r="AD1" s="9" t="s">
-        <v>230</v>
       </c>
       <c r="AE1" s="11" t="s">
         <v>22</v>
@@ -1378,28 +1378,28 @@
         <v>31</v>
       </c>
       <c r="AO1" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="AP1" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="AQ1" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="AR1" s="11" t="s">
         <v>165</v>
       </c>
-      <c r="AP1" s="11" t="s">
+      <c r="AS1" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="AQ1" s="11" t="s">
+      <c r="AT1" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="AR1" s="11" t="s">
+      <c r="AU1" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="AS1" s="11" t="s">
+      <c r="AV1" s="11" t="s">
         <v>169</v>
-      </c>
-      <c r="AT1" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="AU1" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="AV1" s="11" t="s">
-        <v>172</v>
       </c>
       <c r="AW1" s="11" t="s">
         <v>32</v>
@@ -1429,28 +1429,28 @@
         <v>40</v>
       </c>
       <c r="BF1" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="BG1" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="BH1" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="BI1" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="BG1" s="9" t="s">
+      <c r="BJ1" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="BH1" s="9" t="s">
+      <c r="BK1" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="BI1" s="9" t="s">
+      <c r="BL1" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="BJ1" s="9" t="s">
+      <c r="BM1" s="9" t="s">
         <v>177</v>
-      </c>
-      <c r="BK1" s="9" t="s">
-        <v>178</v>
-      </c>
-      <c r="BL1" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="BM1" s="9" t="s">
-        <v>180</v>
       </c>
       <c r="BN1" s="9" t="s">
         <v>41</v>
@@ -1486,34 +1486,34 @@
         <v>51</v>
       </c>
       <c r="BY1" s="11" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="BZ1" s="11" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="CA1" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="CB1" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="CC1" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="CD1" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="CB1" s="11" t="s">
+      <c r="CE1" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="CC1" s="11" t="s">
+      <c r="CF1" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="CD1" s="11" t="s">
+      <c r="CG1" s="11" t="s">
         <v>184</v>
       </c>
-      <c r="CE1" s="11" t="s">
+      <c r="CH1" s="11" t="s">
         <v>185</v>
-      </c>
-      <c r="CF1" s="11" t="s">
-        <v>186</v>
-      </c>
-      <c r="CG1" s="11" t="s">
-        <v>187</v>
-      </c>
-      <c r="CH1" s="11" t="s">
-        <v>188</v>
       </c>
       <c r="CI1" s="9" t="s">
         <v>52</v>
@@ -1534,1208 +1534,1208 @@
         <v>57</v>
       </c>
       <c r="CO1" s="9" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="CP1" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="CQ1" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="CR1" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="CS1" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="CT1" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="CU1" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="CV1" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="CW1" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="CX1" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="CY1" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="CZ1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="DA1" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="DB1" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="DC1" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="DD1" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="DE1" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="DF1" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="DG1" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="DH1" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="DI1" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="DJ1" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="DK1" s="15" t="s">
+        <v>233</v>
+      </c>
+      <c r="DL1" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="DM1" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="DN1" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="DO1" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="DP1" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="DQ1" s="15" t="s">
         <v>234</v>
       </c>
-      <c r="CQ1" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="CR1" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="CS1" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="CT1" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="CU1" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="CV1" s="9" t="s">
-        <v>194</v>
-      </c>
-      <c r="CW1" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="CX1" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="CY1" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="CZ1" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="DA1" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="DB1" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="DC1" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="DD1" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="DE1" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="DF1" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="DG1" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="DH1" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="DI1" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="DJ1" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="DK1" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="DL1" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="DM1" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="DN1" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="DO1" s="15" t="s">
+      <c r="DR1" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="DP1" s="15" t="s">
+      <c r="DS1" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="DQ1" s="15" t="s">
+      <c r="DT1" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="DR1" s="15" t="s">
+      <c r="DU1" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="DS1" s="15" t="s">
+      <c r="DV1" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="DT1" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="DU1" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="DV1" s="15" t="s">
-        <v>81</v>
-      </c>
       <c r="DW1" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="DX1" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="DY1" s="4" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="DZ1" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:130" s="3" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="M2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="N2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="O2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="P2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="R2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="S2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="T2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="U2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="V2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="W2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="X2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="Z2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="AA2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="AB2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="AC2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="AD2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="AE2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AF2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AG2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AH2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="AI2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="AJ2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="AK2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AL2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AM2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AN2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AO2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AP2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AQ2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AR2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AS2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AT2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AU2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AV2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AW2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AX2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AY2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="AZ2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="BA2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="BB2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BC2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BD2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BE2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BF2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BG2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BH2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BI2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BJ2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BK2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BL2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BM2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BN2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BO2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BP2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BQ2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BR2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="BS2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="BT2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="BU2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="BV2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="BW2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="BX2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="BY2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="BZ2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="CA2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="CB2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="CC2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="CD2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="CE2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="CF2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="CG2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="CH2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="CI2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CJ2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CK2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CL2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CM2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CN2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CO2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CP2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CQ2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CR2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CS2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CT2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CU2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CV2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CW2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CX2" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="CY2" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="CZ2" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="DA2" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="DB2" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="DC2" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="DD2" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="DE2" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="DF2" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="DG2" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="DH2" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="DI2" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="DJ2" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="DK2" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="G2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="H2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="I2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="J2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="K2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="L2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="M2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="N2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="O2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="P2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="R2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="S2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="T2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="U2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="V2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="W2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="X2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="Y2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="Z2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="AA2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="AB2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="AC2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="AD2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="AE2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AF2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AG2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AH2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="AI2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="AJ2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="AK2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AL2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AN2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AO2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AP2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AQ2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AR2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AS2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AT2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AU2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AV2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AW2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AX2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AY2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="AZ2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="BA2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="BB2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BC2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BD2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BE2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BF2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BG2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BH2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BI2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BJ2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BK2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BL2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BM2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BN2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BO2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BP2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BQ2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BR2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="BS2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="BT2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="BU2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="BV2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="BW2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="BX2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="BY2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="BZ2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="CA2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="CB2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="CC2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="CD2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="CE2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="CF2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="CG2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="CH2" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="CI2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CJ2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CK2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CL2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CM2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CN2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CO2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CP2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CQ2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CR2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CS2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CT2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CU2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CV2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CW2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CX2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="CY2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="CZ2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="DA2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="DB2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="DC2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="DD2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="DE2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="DF2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="DG2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="DH2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="DI2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="DJ2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="DK2" s="16" t="s">
-        <v>87</v>
-      </c>
       <c r="DL2" s="16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="DM2" s="16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="DN2" s="16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="DO2" s="16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="DP2" s="16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="DQ2" s="16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="DR2" s="16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="DS2" s="16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="DT2" s="16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="DU2" s="16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="DV2" s="16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="DW2" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="DX2" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="DY2" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="DZ2" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:130" s="3" customFormat="1" ht="299" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F3" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="G3" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="L3" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="M3" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="N3" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="F3" s="11" t="s">
+      <c r="O3" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="P3" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="Q3" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="R3" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="S3" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="T3" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="U3" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="V3" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="I3" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="J3" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="K3" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="L3" s="11" t="s">
+      <c r="W3" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="X3" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="Y3" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="Z3" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="AA3" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="AB3" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="AC3" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="AD3" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="AE3" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="M3" s="11" t="s">
+      <c r="AF3" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="AG3" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="AH3" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="N3" s="11" t="s">
+      <c r="AI3" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="O3" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="P3" s="11" t="s">
-        <v>222</v>
-      </c>
-      <c r="Q3" s="11" t="s">
-        <v>225</v>
-      </c>
-      <c r="R3" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="S3" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="T3" s="9" t="s">
+      <c r="AJ3" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="U3" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="V3" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="W3" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="X3" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="Y3" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="Z3" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="AA3" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="AB3" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="AC3" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="AD3" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="AE3" s="11" t="s">
+      <c r="AK3" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="AF3" s="11" t="s">
+      <c r="AL3" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="AG3" s="11" t="s">
+      <c r="AM3" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="AH3" s="9" t="s">
+      <c r="AN3" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="AO3" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="AP3" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="AQ3" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="AR3" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="AS3" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="AT3" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="AU3" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="AV3" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="AW3" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="AX3" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="AY3" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="AZ3" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="BA3" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="BB3" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="AI3" s="9" t="s">
+      <c r="BC3" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="AJ3" s="9" t="s">
+      <c r="BD3" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="AK3" s="11" t="s">
+      <c r="BE3" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="AL3" s="11" t="s">
+      <c r="BF3" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="BG3" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="BH3" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="BI3" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="BJ3" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="BK3" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="BL3" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="BM3" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="BN3" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="AM3" s="11" t="s">
+      <c r="BO3" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="AN3" s="11" t="s">
+      <c r="BP3" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="AO3" s="11" t="s">
-        <v>197</v>
-      </c>
-      <c r="AP3" s="11" t="s">
-        <v>200</v>
-      </c>
-      <c r="AQ3" s="11" t="s">
-        <v>199</v>
-      </c>
-      <c r="AR3" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="AS3" s="11" t="s">
-        <v>201</v>
-      </c>
-      <c r="AT3" s="11" t="s">
-        <v>202</v>
-      </c>
-      <c r="AU3" s="11" t="s">
+      <c r="BQ3" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="BR3" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="BS3" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="BT3" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="BU3" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="BV3" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="BW3" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="BX3" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="BY3" s="11" t="s">
+        <v>213</v>
+      </c>
+      <c r="BZ3" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="CA3" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="AV3" s="11" t="s">
+      <c r="CB3" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="CC3" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="AW3" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="AX3" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="AY3" s="11" t="s">
+      <c r="CD3" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="CE3" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="CF3" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="CG3" s="11" t="s">
+        <v>209</v>
+      </c>
+      <c r="CH3" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="CI3" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="AZ3" s="11" t="s">
+      <c r="CJ3" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="BA3" s="11" t="s">
+      <c r="CK3" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="BB3" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="BC3" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="BD3" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="BE3" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="BF3" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="BG3" s="9" t="s">
-        <v>200</v>
-      </c>
-      <c r="BH3" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="BI3" s="9" t="s">
-        <v>198</v>
-      </c>
-      <c r="BJ3" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="BK3" s="9" t="s">
-        <v>202</v>
-      </c>
-      <c r="BL3" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="BM3" s="9" t="s">
+      <c r="CL3" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="CM3" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="CN3" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="CO3" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="CP3" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="CQ3" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="CR3" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="BN3" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="BO3" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="BP3" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="BQ3" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="BR3" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="BS3" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="BT3" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="BU3" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="BV3" s="11" t="s">
+      <c r="CS3" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="CT3" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="CU3" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="CV3" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="CW3" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="CX3" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="CY3" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="BW3" s="11" t="s">
+      <c r="CZ3" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="BX3" s="11" t="s">
+      <c r="DA3" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="BY3" s="11" t="s">
-        <v>216</v>
-      </c>
-      <c r="BZ3" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="CA3" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="CB3" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="CC3" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="CD3" s="11" t="s">
-        <v>209</v>
-      </c>
-      <c r="CE3" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="CF3" s="11" t="s">
-        <v>211</v>
-      </c>
-      <c r="CG3" s="11" t="s">
-        <v>212</v>
-      </c>
-      <c r="CH3" s="11" t="s">
-        <v>213</v>
-      </c>
-      <c r="CI3" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="CJ3" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="CK3" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="CL3" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="CM3" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="CN3" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="CO3" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="CP3" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="CQ3" s="9" t="s">
-        <v>214</v>
-      </c>
-      <c r="CR3" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="CS3" s="9" t="s">
-        <v>208</v>
-      </c>
-      <c r="CT3" s="9" t="s">
-        <v>209</v>
-      </c>
-      <c r="CU3" s="9" t="s">
-        <v>210</v>
-      </c>
-      <c r="CV3" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="CW3" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="CX3" s="9" t="s">
-        <v>213</v>
-      </c>
-      <c r="CY3" s="7" t="s">
+      <c r="DB3" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="CZ3" s="7" t="s">
+      <c r="DC3" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="DA3" s="7" t="s">
+      <c r="DD3" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="DB3" s="7" t="s">
+      <c r="DE3" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="DC3" s="7" t="s">
+      <c r="DF3" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="DD3" s="7" t="s">
+      <c r="DG3" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="DE3" s="7" t="s">
+      <c r="DH3" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="DF3" s="7" t="s">
+      <c r="DI3" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="DG3" s="7" t="s">
+      <c r="DJ3" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="DH3" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="DI3" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="DJ3" s="7" t="s">
-        <v>124</v>
-      </c>
       <c r="DK3" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="DL3" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="DM3" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="DN3" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="DL3" s="16" t="s">
+      <c r="DO3" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="DM3" s="16" t="s">
+      <c r="DP3" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="DN3" s="16" t="s">
+      <c r="DQ3" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="DR3" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="DO3" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="DP3" s="16" t="s">
+      <c r="DS3" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="DT3" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="DU3" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="DV3" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="DW3" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="DX3" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="DY3" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="DQ3" s="16" t="s">
-        <v>142</v>
-      </c>
-      <c r="DR3" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="DS3" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="DT3" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="DU3" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="DV3" s="16" t="s">
-        <v>147</v>
-      </c>
-      <c r="DW3" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="DX3" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="DY3" s="4" t="s">
+      <c r="DZ3" s="4" t="s">
         <v>150</v>
-      </c>
-      <c r="DZ3" s="4" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:130" s="3" customFormat="1" ht="100.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="L4" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="M4" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="N4" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="O4" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="P4" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="Q4" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="R4" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="S4" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="T4" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="U4" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="V4" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="W4" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="X4" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="Y4" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="Z4" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="AA4" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="AB4" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="AC4" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="AD4" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="AE4" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="AF4" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="F4" s="11" t="s">
+      <c r="AG4" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="AH4" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="AI4" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="AJ4" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="AK4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="AL4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="AM4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="AN4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="AO4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="AS4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="AT4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="AU4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="AV4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW4" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="AX4" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="J4" s="11" t="s">
+      <c r="AY4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="AZ4" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="BA4" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="BB4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BC4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BG4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BH4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BI4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BJ4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BN4" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="K4" s="11" t="s">
+      <c r="BO4" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="L4" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="M4" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="N4" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="O4" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="P4" s="11" t="s">
-        <v>223</v>
-      </c>
-      <c r="Q4" s="11" t="s">
-        <v>226</v>
-      </c>
-      <c r="R4" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="S4" s="11" t="s">
-        <v>141</v>
-      </c>
-      <c r="T4" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="U4" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="V4" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="W4" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="X4" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="Y4" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="Z4" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="AA4" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="AB4" s="9" t="s">
-        <v>163</v>
-      </c>
-      <c r="AC4" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="AD4" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="AE4" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="AF4" s="11" t="s">
+      <c r="BP4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BQ4" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="AG4" s="11" t="s">
+      <c r="BR4" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="AH4" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="AI4" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="AJ4" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="AK4" s="11" t="s">
+      <c r="BS4" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="AL4" s="11" t="s">
+      <c r="BT4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="BU4" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="BV4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="BW4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="BX4" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="BY4" s="11" t="s">
+        <v>214</v>
+      </c>
+      <c r="BZ4" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="CA4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CB4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CC4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CD4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CE4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CI4" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="AM4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="AN4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="AO4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="AP4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="AQ4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="AR4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="AS4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="AT4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="AU4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="AV4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="AW4" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="AX4" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="AY4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="AZ4" s="11" t="s">
+      <c r="CJ4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="CK4" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="CL4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN4" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="BA4" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="BB4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="BC4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="BD4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="BE4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="BF4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="BG4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="BH4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="BI4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="BJ4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="BK4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="BL4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="BM4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="BN4" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="BO4" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="BP4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="BQ4" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="BR4" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="BS4" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="BT4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="BU4" s="11" t="s">
-        <v>219</v>
-      </c>
-      <c r="BV4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="BW4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="BX4" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="BY4" s="11" t="s">
-        <v>217</v>
-      </c>
-      <c r="BZ4" s="11" t="s">
-        <v>233</v>
-      </c>
-      <c r="CA4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="CB4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="CC4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="CD4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="CE4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="CF4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="CG4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="CH4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="CI4" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="CJ4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="CK4" s="9" t="s">
-        <v>218</v>
-      </c>
-      <c r="CL4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="CM4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="CN4" s="9" t="s">
-        <v>135</v>
-      </c>
       <c r="CO4" s="9" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="CP4" s="9" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="CQ4" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="CR4" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="CS4" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="CT4" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="CU4" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="CV4" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="CW4" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="CX4" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="CY4" s="7"/>
       <c r="CZ4" s="7"/>

</xml_diff>

<commit_message>
Edited variable defs and added June RQ8 Table
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/Research/variables/Variable Definitions RQ8_PH2_APR26.xlsx
+++ b/dashboard-ui/src/components/Research/variables/Variable Definitions RQ8_PH2_APR26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gary.cheng_cn\Projects\itm-evaluation-dashboard\dashboard-ui\src\components\Research\variables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C120C1-3157-4CC0-8B81-B1DDAF42F4E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{710F2D95-9BEA-42AF-9B4C-CDC9E00F94DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RQ8" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="237">
   <si>
     <t>Variables</t>
   </si>
@@ -579,9 +579,6 @@
   </si>
   <si>
     <t>Desert Patient{N}_treat_repeat_hits_required</t>
-  </si>
-  <si>
-    <t>Desert Patient[{N}_treat_repeat_false_alarms_required</t>
   </si>
   <si>
     <t>Desert Patient{N}_treat_hits_w_supp</t>
@@ -767,6 +764,15 @@
   </si>
   <si>
     <t>AF_intercept_Urban</t>
+  </si>
+  <si>
+    <t>Desert Patient{N}_treat_repeat_false_alarms_required</t>
+  </si>
+  <si>
+    <t>Urban Probe_PS1_Actions</t>
+  </si>
+  <si>
+    <t>List of moderator buttons the participant selected in response to the initial personal-safety inject</t>
   </si>
 </sst>
 </file>
@@ -1207,7 +1213,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:DZ6"/>
+  <dimension ref="A1:EA6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="16.7265625" style="2" bestFit="1" customWidth="1"/>
@@ -1221,42 +1227,42 @@
     <col min="20" max="25" width="12.453125" style="10" bestFit="1" customWidth="1"/>
     <col min="26" max="27" width="13" style="10" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="12.453125" style="10" bestFit="1" customWidth="1"/>
-    <col min="29" max="30" width="12.453125" style="10" customWidth="1"/>
-    <col min="31" max="33" width="16.7265625" style="12" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="16.7265625" style="10" bestFit="1" customWidth="1"/>
-    <col min="37" max="39" width="16.7265625" style="12" bestFit="1" customWidth="1"/>
-    <col min="40" max="48" width="16.7265625" style="12" customWidth="1"/>
-    <col min="49" max="53" width="13" style="12" bestFit="1" customWidth="1"/>
-    <col min="54" max="57" width="16.7265625" style="10" bestFit="1" customWidth="1"/>
-    <col min="58" max="65" width="16.7265625" style="10" customWidth="1"/>
-    <col min="66" max="70" width="13" style="10" bestFit="1" customWidth="1"/>
-    <col min="71" max="76" width="13" style="12" bestFit="1" customWidth="1"/>
-    <col min="77" max="86" width="13" style="12" customWidth="1"/>
-    <col min="87" max="92" width="13" style="10" bestFit="1" customWidth="1"/>
-    <col min="93" max="102" width="13" style="10" customWidth="1"/>
-    <col min="103" max="103" width="87.7265625" style="8" customWidth="1"/>
-    <col min="104" max="105" width="73" style="8" bestFit="1" customWidth="1"/>
-    <col min="106" max="106" width="38.54296875" style="6" customWidth="1"/>
-    <col min="107" max="107" width="34.7265625" style="6" customWidth="1"/>
-    <col min="108" max="108" width="73" style="8" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="32.54296875" style="6" customWidth="1"/>
-    <col min="110" max="114" width="32.26953125" style="6" customWidth="1"/>
-    <col min="115" max="115" width="87.7265625" style="17" customWidth="1"/>
-    <col min="116" max="117" width="73" style="17" bestFit="1" customWidth="1"/>
-    <col min="118" max="118" width="38.54296875" style="15" customWidth="1"/>
-    <col min="119" max="119" width="34.7265625" style="15" customWidth="1"/>
-    <col min="120" max="120" width="73" style="17" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="87.7265625" style="17" customWidth="1"/>
-    <col min="122" max="123" width="73" style="17" bestFit="1" customWidth="1"/>
-    <col min="124" max="124" width="38.54296875" style="15" customWidth="1"/>
-    <col min="125" max="125" width="34.7265625" style="15" customWidth="1"/>
-    <col min="126" max="126" width="73" style="17" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="14.7265625" style="5" customWidth="1"/>
-    <col min="128" max="128" width="15.26953125" style="5" customWidth="1"/>
-    <col min="129" max="130" width="9.1796875" style="5"/>
+    <col min="29" max="31" width="12.453125" style="10" customWidth="1"/>
+    <col min="32" max="34" width="16.7265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="35" max="37" width="16.7265625" style="10" bestFit="1" customWidth="1"/>
+    <col min="38" max="40" width="16.7265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="41" max="49" width="16.7265625" style="12" customWidth="1"/>
+    <col min="50" max="54" width="13" style="12" bestFit="1" customWidth="1"/>
+    <col min="55" max="58" width="16.7265625" style="10" bestFit="1" customWidth="1"/>
+    <col min="59" max="66" width="16.7265625" style="10" customWidth="1"/>
+    <col min="67" max="71" width="13" style="10" bestFit="1" customWidth="1"/>
+    <col min="72" max="77" width="13" style="12" bestFit="1" customWidth="1"/>
+    <col min="78" max="87" width="13" style="12" customWidth="1"/>
+    <col min="88" max="93" width="13" style="10" bestFit="1" customWidth="1"/>
+    <col min="94" max="103" width="13" style="10" customWidth="1"/>
+    <col min="104" max="104" width="87.7265625" style="8" customWidth="1"/>
+    <col min="105" max="106" width="73" style="8" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="38.54296875" style="6" customWidth="1"/>
+    <col min="108" max="108" width="34.7265625" style="6" customWidth="1"/>
+    <col min="109" max="109" width="73" style="8" bestFit="1" customWidth="1"/>
+    <col min="110" max="110" width="32.54296875" style="6" customWidth="1"/>
+    <col min="111" max="115" width="32.26953125" style="6" customWidth="1"/>
+    <col min="116" max="116" width="87.7265625" style="17" customWidth="1"/>
+    <col min="117" max="118" width="73" style="17" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="38.54296875" style="15" customWidth="1"/>
+    <col min="120" max="120" width="34.7265625" style="15" customWidth="1"/>
+    <col min="121" max="121" width="73" style="17" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="87.7265625" style="17" customWidth="1"/>
+    <col min="123" max="124" width="73" style="17" bestFit="1" customWidth="1"/>
+    <col min="125" max="125" width="38.54296875" style="15" customWidth="1"/>
+    <col min="126" max="126" width="34.7265625" style="15" customWidth="1"/>
+    <col min="127" max="127" width="73" style="17" bestFit="1" customWidth="1"/>
+    <col min="128" max="128" width="14.7265625" style="5" customWidth="1"/>
+    <col min="129" max="129" width="15.26953125" style="5" customWidth="1"/>
+    <col min="130" max="131" width="9.1796875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:130" s="3" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:131" s="3" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1303,10 +1309,10 @@
         <v>12</v>
       </c>
       <c r="P1" s="11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="Q1" s="11" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="R1" s="11" t="s">
         <v>135</v>
@@ -1342,313 +1348,316 @@
         <v>21</v>
       </c>
       <c r="AC1" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AD1" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="AE1" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="AF1" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="AG1" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="AH1" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI1" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="AJ1" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="AK1" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="AL1" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="AM1" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="AN1" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="AO1" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="AP1" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="AQ1" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="AR1" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="AS1" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="AT1" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="AU1" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="AV1" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="AW1" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="AX1" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="AY1" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="AZ1" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="BA1" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="BB1" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="BC1" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="BD1" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="BE1" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="BF1" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="BG1" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="BH1" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="BI1" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="BJ1" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="BK1" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="BL1" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="BM1" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="BN1" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="BO1" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="BP1" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="BQ1" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="BR1" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="BS1" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="BT1" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="BU1" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="BV1" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="BW1" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="BX1" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="BY1" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="BZ1" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="CA1" s="11" t="s">
         <v>227</v>
       </c>
-      <c r="AE1" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="AF1" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="AG1" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="AH1" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="AI1" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="AJ1" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="AK1" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="AL1" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="AM1" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="AN1" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="AO1" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="AP1" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="AQ1" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="AR1" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="AS1" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="AT1" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="AU1" s="11" t="s">
-        <v>168</v>
-      </c>
-      <c r="AV1" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="AW1" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="AX1" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="AY1" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="AZ1" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="BA1" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="BB1" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="BC1" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="BD1" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="BE1" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="BF1" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="BG1" s="9" t="s">
-        <v>171</v>
-      </c>
-      <c r="BH1" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="BI1" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="BJ1" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="BK1" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="BL1" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="BM1" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="BN1" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="BO1" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="BP1" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="BQ1" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="BR1" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="BS1" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="BT1" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="BU1" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="BV1" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="BW1" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="BX1" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="BY1" s="11" t="s">
-        <v>217</v>
-      </c>
-      <c r="BZ1" s="11" t="s">
-        <v>228</v>
-      </c>
-      <c r="CA1" s="11" t="s">
+      <c r="CB1" s="11" t="s">
         <v>178</v>
       </c>
-      <c r="CB1" s="11" t="s">
+      <c r="CC1" s="11" t="s">
         <v>179</v>
       </c>
-      <c r="CC1" s="11" t="s">
+      <c r="CD1" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="CD1" s="11" t="s">
+      <c r="CE1" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="CF1" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="CE1" s="11" t="s">
+      <c r="CG1" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="CF1" s="11" t="s">
+      <c r="CH1" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="CG1" s="11" t="s">
+      <c r="CI1" s="11" t="s">
         <v>184</v>
       </c>
-      <c r="CH1" s="11" t="s">
+      <c r="CJ1" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="CK1" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="CL1" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="CM1" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="CN1" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="CO1" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="CP1" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="CQ1" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="CR1" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="CI1" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="CJ1" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="CK1" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="CL1" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="CM1" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="CN1" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="CO1" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="CP1" s="9" t="s">
+      <c r="CS1" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="CT1" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="CU1" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="CV1" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="CW1" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="CX1" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="CY1" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="CZ1" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="CQ1" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="CR1" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="CS1" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="CT1" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="CU1" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="CV1" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="CW1" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="CX1" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="CY1" s="6" t="s">
+      <c r="DA1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="DB1" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="DC1" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="DD1" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="DE1" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="DF1" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="DG1" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="DH1" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="DI1" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="DJ1" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="DK1" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="DL1" s="15" t="s">
         <v>232</v>
       </c>
-      <c r="CZ1" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="DA1" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="DB1" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="DC1" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="DD1" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="DE1" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="DF1" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="DG1" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="DH1" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="DI1" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="DJ1" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="DK1" s="15" t="s">
+      <c r="DM1" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="DN1" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="DO1" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="DP1" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="DQ1" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="DR1" s="15" t="s">
         <v>233</v>
       </c>
-      <c r="DL1" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="DM1" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="DN1" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="DO1" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="DP1" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="DQ1" s="15" t="s">
-        <v>234</v>
-      </c>
-      <c r="DR1" s="15" t="s">
+      <c r="DS1" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="DS1" s="15" t="s">
+      <c r="DT1" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="DT1" s="15" t="s">
+      <c r="DU1" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="DU1" s="15" t="s">
+      <c r="DV1" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="DV1" s="15" t="s">
+      <c r="DW1" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="DW1" s="4" t="s">
+      <c r="DX1" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="DX1" s="4" t="s">
+      <c r="DY1" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="DY1" s="4" t="s">
+      <c r="DZ1" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="DZ1" s="4" t="s">
+      <c r="EA1" s="4" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="2" spans="1:130" s="3" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:131" s="3" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>79</v>
       </c>
@@ -1739,7 +1748,7 @@
       <c r="AD2" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="AE2" s="11" t="s">
+      <c r="AE2" s="9" t="s">
         <v>82</v>
       </c>
       <c r="AF2" s="11" t="s">
@@ -1748,7 +1757,7 @@
       <c r="AG2" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="AH2" s="9" t="s">
+      <c r="AH2" s="11" t="s">
         <v>82</v>
       </c>
       <c r="AI2" s="9" t="s">
@@ -1757,7 +1766,7 @@
       <c r="AJ2" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="AK2" s="11" t="s">
+      <c r="AK2" s="9" t="s">
         <v>82</v>
       </c>
       <c r="AL2" s="11" t="s">
@@ -1808,7 +1817,7 @@
       <c r="BA2" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="BB2" s="9" t="s">
+      <c r="BB2" s="11" t="s">
         <v>82</v>
       </c>
       <c r="BC2" s="9" t="s">
@@ -1859,7 +1868,7 @@
       <c r="BR2" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="BS2" s="11" t="s">
+      <c r="BS2" s="9" t="s">
         <v>82</v>
       </c>
       <c r="BT2" s="11" t="s">
@@ -1907,7 +1916,7 @@
       <c r="CH2" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="CI2" s="9" t="s">
+      <c r="CI2" s="11" t="s">
         <v>82</v>
       </c>
       <c r="CJ2" s="9" t="s">
@@ -1955,8 +1964,8 @@
       <c r="CX2" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="CY2" s="7" t="s">
-        <v>83</v>
+      <c r="CY2" s="9" t="s">
+        <v>82</v>
       </c>
       <c r="CZ2" s="7" t="s">
         <v>83</v>
@@ -1991,8 +2000,8 @@
       <c r="DJ2" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="DK2" s="16" t="s">
-        <v>84</v>
+      <c r="DK2" s="7" t="s">
+        <v>83</v>
       </c>
       <c r="DL2" s="16" t="s">
         <v>84</v>
@@ -2027,8 +2036,8 @@
       <c r="DV2" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="DW2" s="4" t="s">
-        <v>146</v>
+      <c r="DW2" s="16" t="s">
+        <v>84</v>
       </c>
       <c r="DX2" s="4" t="s">
         <v>146</v>
@@ -2039,8 +2048,11 @@
       <c r="DZ2" s="4" t="s">
         <v>146</v>
       </c>
+      <c r="EA2" s="4" t="s">
+        <v>146</v>
+      </c>
     </row>
-    <row r="3" spans="1:130" s="3" customFormat="1" ht="299" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:131" s="3" customFormat="1" ht="299" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>85</v>
       </c>
@@ -2087,10 +2099,10 @@
         <v>133</v>
       </c>
       <c r="P3" s="11" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="Q3" s="11" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="R3" s="11" t="s">
         <v>90</v>
@@ -2126,46 +2138,46 @@
         <v>90</v>
       </c>
       <c r="AC3" s="9" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="AD3" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="AE3" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="AE3" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="AF3" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="AF3" s="11" t="s">
+      <c r="AG3" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="AG3" s="11" t="s">
+      <c r="AH3" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="AH3" s="9" t="s">
+      <c r="AI3" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="AI3" s="9" t="s">
+      <c r="AJ3" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="AJ3" s="9" t="s">
+      <c r="AK3" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="AK3" s="11" t="s">
+      <c r="AL3" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="AL3" s="11" t="s">
+      <c r="AM3" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="AM3" s="11" t="s">
+      <c r="AN3" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="AN3" s="11" t="s">
+      <c r="AO3" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="AO3" s="11" t="s">
-        <v>194</v>
-      </c>
       <c r="AP3" s="11" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="AQ3" s="11" t="s">
         <v>196</v>
@@ -2174,49 +2186,49 @@
         <v>195</v>
       </c>
       <c r="AS3" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="AT3" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="AU3" s="11" t="s">
         <v>198</v>
       </c>
-      <c r="AT3" s="11" t="s">
+      <c r="AV3" s="11" t="s">
         <v>199</v>
       </c>
-      <c r="AU3" s="11" t="s">
-        <v>200</v>
-      </c>
-      <c r="AV3" s="11" t="s">
-        <v>202</v>
-      </c>
       <c r="AW3" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="AX3" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="AX3" s="11" t="s">
+      <c r="AY3" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="AY3" s="11" t="s">
+      <c r="AZ3" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="AZ3" s="11" t="s">
+      <c r="BA3" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="BA3" s="11" t="s">
+      <c r="BB3" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="BB3" s="9" t="s">
+      <c r="BC3" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="BC3" s="9" t="s">
+      <c r="BD3" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="BD3" s="9" t="s">
+      <c r="BE3" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="BE3" s="9" t="s">
+      <c r="BF3" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="BF3" s="9" t="s">
-        <v>194</v>
-      </c>
       <c r="BG3" s="9" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="BH3" s="9" t="s">
         <v>196</v>
@@ -2225,214 +2237,217 @@
         <v>195</v>
       </c>
       <c r="BJ3" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="BK3" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="BL3" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="BK3" s="9" t="s">
+      <c r="BM3" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="BL3" s="9" t="s">
+      <c r="BN3" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="BM3" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="BN3" s="9" t="s">
+      <c r="BO3" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="BO3" s="9" t="s">
+      <c r="BP3" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="BP3" s="9" t="s">
+      <c r="BQ3" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="BQ3" s="9" t="s">
+      <c r="BR3" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="BR3" s="9" t="s">
+      <c r="BS3" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="BS3" s="11" t="s">
+      <c r="BT3" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="BT3" s="11" t="s">
+      <c r="BU3" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="BU3" s="11" t="s">
+      <c r="BV3" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="BV3" s="11" t="s">
+      <c r="BW3" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="BW3" s="11" t="s">
+      <c r="BX3" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="BX3" s="11" t="s">
+      <c r="BY3" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="BY3" s="11" t="s">
-        <v>213</v>
-      </c>
       <c r="BZ3" s="11" t="s">
-        <v>229</v>
+        <v>212</v>
       </c>
       <c r="CA3" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="CB3" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="CC3" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="CB3" s="11" t="s">
+      <c r="CD3" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="CC3" s="11" t="s">
+      <c r="CE3" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="CD3" s="11" t="s">
+      <c r="CF3" s="11" t="s">
         <v>206</v>
       </c>
-      <c r="CE3" s="11" t="s">
+      <c r="CG3" s="11" t="s">
         <v>207</v>
       </c>
-      <c r="CF3" s="11" t="s">
+      <c r="CH3" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="CG3" s="11" t="s">
+      <c r="CI3" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="CH3" s="11" t="s">
+      <c r="CJ3" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="CK3" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="CL3" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="CM3" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="CN3" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="CO3" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="CP3" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="CQ3" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="CR3" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="CI3" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="CJ3" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="CK3" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="CL3" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="CM3" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="CN3" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="CO3" s="9" t="s">
-        <v>213</v>
-      </c>
-      <c r="CP3" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="CQ3" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="CR3" s="9" t="s">
+      <c r="CS3" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="CT3" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="CS3" s="9" t="s">
+      <c r="CU3" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="CT3" s="9" t="s">
+      <c r="CV3" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="CU3" s="9" t="s">
+      <c r="CW3" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="CV3" s="9" t="s">
+      <c r="CX3" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="CW3" s="9" t="s">
+      <c r="CY3" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="CX3" s="9" t="s">
-        <v>210</v>
-      </c>
-      <c r="CY3" s="7" t="s">
+      <c r="CZ3" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="CZ3" s="7" t="s">
+      <c r="DA3" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="DA3" s="7" t="s">
+      <c r="DB3" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="DB3" s="7" t="s">
+      <c r="DC3" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="DC3" s="7" t="s">
+      <c r="DD3" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="DD3" s="7" t="s">
+      <c r="DE3" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="DE3" s="7" t="s">
+      <c r="DF3" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="DF3" s="7" t="s">
+      <c r="DG3" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="DG3" s="7" t="s">
+      <c r="DH3" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="DH3" s="7" t="s">
+      <c r="DI3" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="DI3" s="7" t="s">
+      <c r="DJ3" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="DJ3" s="7" t="s">
+      <c r="DK3" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="DK3" s="16" t="s">
+      <c r="DL3" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="DL3" s="16" t="s">
+      <c r="DM3" s="16" t="s">
         <v>140</v>
       </c>
-      <c r="DM3" s="16" t="s">
+      <c r="DN3" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="DN3" s="16" t="s">
+      <c r="DO3" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="DO3" s="16" t="s">
+      <c r="DP3" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="DP3" s="16" t="s">
+      <c r="DQ3" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="DQ3" s="16" t="s">
+      <c r="DR3" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="DR3" s="16" t="s">
+      <c r="DS3" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="DS3" s="16" t="s">
+      <c r="DT3" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="DT3" s="16" t="s">
+      <c r="DU3" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="DU3" s="16" t="s">
+      <c r="DV3" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="DV3" s="16" t="s">
+      <c r="DW3" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="DW3" s="4" t="s">
+      <c r="DX3" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="DX3" s="4" t="s">
+      <c r="DY3" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="DY3" s="4" t="s">
+      <c r="DZ3" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="DZ3" s="4" t="s">
+      <c r="EA3" s="4" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="4" spans="1:130" s="3" customFormat="1" ht="100.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:131" s="3" customFormat="1" ht="100.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>122</v>
       </c>
@@ -2477,10 +2492,10 @@
         <v>134</v>
       </c>
       <c r="P4" s="11" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="Q4" s="11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="R4" s="11" t="s">
         <v>137</v>
@@ -2516,32 +2531,32 @@
         <v>160</v>
       </c>
       <c r="AC4" s="9" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AD4" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="AE4" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="AE4" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="AF4" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="AF4" s="11" t="s">
+      <c r="AG4" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="AG4" s="11" t="s">
+      <c r="AH4" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="AH4" s="9" t="s">
+      <c r="AI4" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="AI4" s="9" t="s">
+      <c r="AJ4" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="AJ4" s="9" t="s">
+      <c r="AK4" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="AK4" s="11" t="s">
-        <v>128</v>
-      </c>
       <c r="AL4" s="11" t="s">
         <v>128</v>
       </c>
@@ -2576,23 +2591,23 @@
         <v>128</v>
       </c>
       <c r="AW4" s="11" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AX4" s="11" t="s">
         <v>127</v>
       </c>
       <c r="AY4" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AZ4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="BA4" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="BA4" s="11" t="s">
+      <c r="BB4" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="BB4" s="9" t="s">
-        <v>128</v>
-      </c>
       <c r="BC4" s="9" t="s">
         <v>128</v>
       </c>
@@ -2627,94 +2642,94 @@
         <v>128</v>
       </c>
       <c r="BN4" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="BO4" s="9" t="s">
         <v>127</v>
       </c>
       <c r="BP4" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="BQ4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR4" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="BR4" s="9" t="s">
+      <c r="BS4" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="BS4" s="11" t="s">
+      <c r="BT4" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="BT4" s="11" t="s">
-        <v>128</v>
-      </c>
       <c r="BU4" s="11" t="s">
-        <v>216</v>
+        <v>128</v>
       </c>
       <c r="BV4" s="11" t="s">
-        <v>128</v>
+        <v>215</v>
       </c>
       <c r="BW4" s="11" t="s">
         <v>128</v>
       </c>
       <c r="BX4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY4" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="BY4" s="11" t="s">
+      <c r="BZ4" s="11" t="s">
+        <v>213</v>
+      </c>
+      <c r="CA4" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="CB4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CC4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CD4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CE4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CI4" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="CJ4" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="CK4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="CL4" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="BZ4" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="CA4" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="CB4" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="CC4" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="CD4" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="CE4" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="CF4" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="CG4" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="CH4" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="CI4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="CJ4" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="CK4" s="9" t="s">
-        <v>215</v>
-      </c>
-      <c r="CL4" s="9" t="s">
-        <v>128</v>
-      </c>
       <c r="CM4" s="9" t="s">
         <v>128</v>
       </c>
       <c r="CN4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO4" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="CO4" s="9" t="s">
-        <v>214</v>
-      </c>
       <c r="CP4" s="9" t="s">
-        <v>230</v>
+        <v>213</v>
       </c>
       <c r="CQ4" s="9" t="s">
-        <v>128</v>
+        <v>229</v>
       </c>
       <c r="CR4" s="9" t="s">
         <v>128</v>
@@ -2737,7 +2752,9 @@
       <c r="CX4" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="CY4" s="7"/>
+      <c r="CY4" s="9" t="s">
+        <v>128</v>
+      </c>
       <c r="CZ4" s="7"/>
       <c r="DA4" s="7"/>
       <c r="DB4" s="7"/>
@@ -2749,7 +2766,7 @@
       <c r="DH4" s="7"/>
       <c r="DI4" s="7"/>
       <c r="DJ4" s="7"/>
-      <c r="DK4" s="16"/>
+      <c r="DK4" s="7"/>
       <c r="DL4" s="16"/>
       <c r="DM4" s="16"/>
       <c r="DN4" s="16"/>
@@ -2761,13 +2778,13 @@
       <c r="DT4" s="16"/>
       <c r="DU4" s="16"/>
       <c r="DV4" s="16"/>
-      <c r="DW4" s="4"/>
+      <c r="DW4" s="16"/>
       <c r="DX4" s="4"/>
       <c r="DY4" s="4"/>
       <c r="DZ4" s="4"/>
+      <c r="EA4" s="4"/>
     </row>
-    <row r="5" spans="1:130" x14ac:dyDescent="0.35">
-      <c r="CY5" s="7"/>
+    <row r="5" spans="1:131" x14ac:dyDescent="0.35">
       <c r="CZ5" s="7"/>
       <c r="DA5" s="7"/>
       <c r="DB5" s="7"/>
@@ -2779,7 +2796,7 @@
       <c r="DH5" s="7"/>
       <c r="DI5" s="7"/>
       <c r="DJ5" s="7"/>
-      <c r="DK5" s="16"/>
+      <c r="DK5" s="7"/>
       <c r="DL5" s="16"/>
       <c r="DM5" s="16"/>
       <c r="DN5" s="16"/>
@@ -2791,9 +2808,9 @@
       <c r="DT5" s="16"/>
       <c r="DU5" s="16"/>
       <c r="DV5" s="16"/>
+      <c r="DW5" s="16"/>
     </row>
-    <row r="6" spans="1:130" x14ac:dyDescent="0.35">
-      <c r="CY6" s="7"/>
+    <row r="6" spans="1:131" x14ac:dyDescent="0.35">
       <c r="CZ6" s="7"/>
       <c r="DA6" s="7"/>
       <c r="DB6" s="7"/>
@@ -2805,7 +2822,7 @@
       <c r="DH6" s="7"/>
       <c r="DI6" s="7"/>
       <c r="DJ6" s="7"/>
-      <c r="DK6" s="16"/>
+      <c r="DK6" s="7"/>
       <c r="DL6" s="16"/>
       <c r="DM6" s="16"/>
       <c r="DN6" s="16"/>
@@ -2817,6 +2834,7 @@
       <c r="DT6" s="16"/>
       <c r="DU6" s="16"/>
       <c r="DV6" s="16"/>
+      <c r="DW6" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>